<commit_message>
Module Produits et Catalogue (iteration 3)
Cote vendeur :
- Espace /vendeur/produits (reserve aux vendeurs approuves) : liste,
  creation, modification, publication/depublication, suppression
- Formulaire produit : 3 a 10 photos vers Storage (previsualisation,
  photo principale, reordonnancement), prix FCFA, prix de gros B2B,
  stock, quantite minimum, poids, delai de preparation, pays d origine
- Nettoyage des fichiers Storage a la suppression des images

Catalogue public :
- 8 categories / 30 sous-categories (drizzle/seed-categories.sql)
- /produits : recherche, filtres (categorie, prix min/max, en stock),
  tri (recents, prix), pagination 12/page
- /produits/[id] : galerie cliquable, prix de gros, vendeur verifie
- Accueil marketplace : categories + nouveautes + en-tete avec recherche

Suivi : 33 fonctionnalites passees en Realise, 2 en Partiel (paliers
de prix, devises) dans Explosion du projet - MAJ.xlsx

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Explosion du projet - MAJ.xlsx
+++ b/docs/Explosion du projet - MAJ.xlsx
@@ -2753,9 +2753,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F51" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F51" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G51" s="34" t="inlineStr">
+        <is>
+          <t>Itération 3</t>
         </is>
       </c>
     </row>
@@ -2783,9 +2788,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F52" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F52" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G52" s="34" t="inlineStr">
+        <is>
+          <t>Itération 3</t>
         </is>
       </c>
     </row>
@@ -2813,9 +2823,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F53" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F53" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G53" s="34" t="inlineStr">
+        <is>
+          <t>Itération 3</t>
         </is>
       </c>
     </row>
@@ -2843,9 +2858,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F54" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F54" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G54" s="34" t="inlineStr">
+        <is>
+          <t>Itération 3</t>
         </is>
       </c>
     </row>
@@ -2873,9 +2893,14 @@
           <t>Moyenne</t>
         </is>
       </c>
-      <c r="F55" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F55" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G55" s="34" t="inlineStr">
+        <is>
+          <t>Itération 3</t>
         </is>
       </c>
     </row>
@@ -2903,9 +2928,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F56" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F56" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G56" s="34" t="inlineStr">
+        <is>
+          <t>Itération 3 — contrôle client et serveur</t>
         </is>
       </c>
     </row>
@@ -2933,9 +2963,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F57" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F57" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G57" s="34" t="inlineStr">
+        <is>
+          <t>Itération 3</t>
         </is>
       </c>
     </row>
@@ -2963,9 +2998,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F58" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F58" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G58" s="34" t="inlineStr">
+        <is>
+          <t>Itération 3 — réordonnancement dans le formulaire</t>
         </is>
       </c>
     </row>
@@ -3023,9 +3063,14 @@
           <t>Moyenne</t>
         </is>
       </c>
-      <c r="F60" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F60" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G60" s="34" t="inlineStr">
+        <is>
+          <t>Itération 3</t>
         </is>
       </c>
     </row>
@@ -3053,9 +3098,14 @@
           <t>Moyenne</t>
         </is>
       </c>
-      <c r="F61" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F61" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G61" s="34" t="inlineStr">
+        <is>
+          <t>Itération 3 — fichiers Storage nettoyés</t>
         </is>
       </c>
     </row>
@@ -3083,9 +3133,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F62" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F62" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G62" s="34" t="inlineStr">
+        <is>
+          <t>Itération 3</t>
         </is>
       </c>
     </row>
@@ -3113,9 +3168,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F63" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F63" s="35" t="inlineStr">
+        <is>
+          <t>🟡 Partiel</t>
+        </is>
+      </c>
+      <c r="G63" s="34" t="inlineStr">
+        <is>
+          <t>Un seul palier pour l'instant (prix de gros)</t>
         </is>
       </c>
     </row>
@@ -3143,9 +3203,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F64" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F64" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G64" s="34" t="inlineStr">
+        <is>
+          <t>Itération 3 — prix + quantité minimum</t>
         </is>
       </c>
     </row>
@@ -3173,9 +3238,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F65" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F65" s="35" t="inlineStr">
+        <is>
+          <t>🟡 Partiel</t>
+        </is>
+      </c>
+      <c r="G65" s="34" t="inlineStr">
+        <is>
+          <t>XOF uniquement pour le MVP</t>
         </is>
       </c>
     </row>
@@ -3203,9 +3273,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F66" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F66" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G66" s="34" t="inlineStr">
+        <is>
+          <t>Itération 3</t>
         </is>
       </c>
     </row>
@@ -3233,9 +3308,14 @@
           <t>Moyenne</t>
         </is>
       </c>
-      <c r="F67" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F67" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G67" s="34" t="inlineStr">
+        <is>
+          <t>Itération 3</t>
         </is>
       </c>
     </row>
@@ -3263,9 +3343,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F68" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F68" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G68" s="34" t="inlineStr">
+        <is>
+          <t>Itération 3 — badge rupture automatique</t>
         </is>
       </c>
     </row>
@@ -3293,9 +3378,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F69" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F69" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G69" s="34" t="inlineStr">
+        <is>
+          <t>Itération 3</t>
         </is>
       </c>
     </row>
@@ -3323,9 +3413,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F70" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F70" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G70" s="34" t="inlineStr">
+        <is>
+          <t>Itération 3</t>
         </is>
       </c>
     </row>
@@ -3413,9 +3508,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F73" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F73" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G73" s="34" t="inlineStr">
+        <is>
+          <t>Itération 3</t>
         </is>
       </c>
     </row>
@@ -3443,9 +3543,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F74" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F74" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G74" s="34" t="inlineStr">
+        <is>
+          <t>Itération 3 — brouillon / en ligne</t>
         </is>
       </c>
     </row>
@@ -3473,9 +3578,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F75" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F75" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G75" s="34" t="inlineStr">
+        <is>
+          <t>Itération 3</t>
         </is>
       </c>
     </row>
@@ -3515,9 +3625,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F77" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F77" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G77" s="34" t="inlineStr">
+        <is>
+          <t>Itération 3 — catégories + nouveautés</t>
         </is>
       </c>
     </row>
@@ -3545,9 +3660,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F78" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F78" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G78" s="34" t="inlineStr">
+        <is>
+          <t>Itération 3</t>
         </is>
       </c>
     </row>
@@ -3575,9 +3695,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F79" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F79" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G79" s="34" t="inlineStr">
+        <is>
+          <t>Itération 3 — 8 catégories, 30 sous-catégories</t>
         </is>
       </c>
     </row>
@@ -3605,9 +3730,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F80" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F80" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G80" s="34" t="inlineStr">
+        <is>
+          <t>Itération 3</t>
         </is>
       </c>
     </row>
@@ -3635,9 +3765,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F81" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F81" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G81" s="34" t="inlineStr">
+        <is>
+          <t>Itération 3 — 12 produits par page</t>
         </is>
       </c>
     </row>
@@ -3665,9 +3800,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F82" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F82" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G82" s="34" t="inlineStr">
+        <is>
+          <t>Itération 3 — dans l'en-tête du site</t>
         </is>
       </c>
     </row>
@@ -3695,9 +3835,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F83" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F83" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G83" s="34" t="inlineStr">
+        <is>
+          <t>Itération 3 — titre et description</t>
         </is>
       </c>
     </row>
@@ -3725,9 +3870,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F84" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F84" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G84" s="34" t="inlineStr">
+        <is>
+          <t>Itération 3</t>
         </is>
       </c>
     </row>
@@ -3755,9 +3905,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F85" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F85" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G85" s="34" t="inlineStr">
+        <is>
+          <t>Itération 3</t>
         </is>
       </c>
     </row>
@@ -3785,9 +3940,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F86" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F86" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G86" s="34" t="inlineStr">
+        <is>
+          <t>Itération 3</t>
         </is>
       </c>
     </row>
@@ -3815,9 +3975,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F87" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F87" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G87" s="34" t="inlineStr">
+        <is>
+          <t>Itération 3 — tri par défaut : plus récents</t>
         </is>
       </c>
     </row>
@@ -3845,9 +4010,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F88" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F88" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G88" s="34" t="inlineStr">
+        <is>
+          <t>Itération 3</t>
         </is>
       </c>
     </row>
@@ -3875,9 +4045,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F89" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F89" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G89" s="34" t="inlineStr">
+        <is>
+          <t>Itération 3</t>
         </is>
       </c>
     </row>
@@ -3905,9 +4080,14 @@
           <t>Moyenne</t>
         </is>
       </c>
-      <c r="F90" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F90" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G90" s="34" t="inlineStr">
+        <is>
+          <t>Itération 3</t>
         </is>
       </c>
     </row>
@@ -18803,8 +18983,6 @@
         </is>
       </c>
     </row>
-    <row r="274"/>
-    <row r="275"/>
     <row r="276" ht="16.3" customHeight="1" s="18">
       <c r="A276" s="24" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Suivi : iteration 5 marquee dans l explosion du projet
87 fonctionnalites MVP realisees, 10 partielles

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Explosion du projet - MAJ.xlsx
+++ b/docs/Explosion du projet - MAJ.xlsx
@@ -1744,9 +1744,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F18" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G18" s="34" t="inlineStr">
+        <is>
+          <t>Itération 5 — page wallet</t>
         </is>
       </c>
     </row>
@@ -1809,14 +1814,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F20" s="35" t="inlineStr">
-        <is>
-          <t>🟡 Partiel</t>
+      <c r="F20" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
         </is>
       </c>
       <c r="G20" s="34" t="inlineStr">
         <is>
-          <t>Statuts visibles ; transitions avec Escrow/Livraison</t>
+          <t>Itération 5 — statuts et transitions complets</t>
         </is>
       </c>
     </row>
@@ -1964,9 +1969,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F25" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F25" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G25" s="34" t="inlineStr">
+        <is>
+          <t>Itération 5 — wallet commun au compte</t>
         </is>
       </c>
     </row>
@@ -1994,14 +2004,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F26" s="35" t="inlineStr">
-        <is>
-          <t>🟡 Partiel</t>
+      <c r="F26" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
         </is>
       </c>
       <c r="G26" s="34" t="inlineStr">
         <is>
-          <t>Liste visible ; traitement avec Escrow</t>
+          <t>Itération 5 — préparation / expédition</t>
         </is>
       </c>
     </row>
@@ -4879,9 +4889,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F114" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F114" s="35" t="inlineStr">
+        <is>
+          <t>🟡 Partiel</t>
+        </is>
+      </c>
+      <c r="G114" s="34" t="inlineStr">
+        <is>
+          <t>Recharge wallet simulée ; agrégateur réel à brancher en prod</t>
         </is>
       </c>
     </row>
@@ -4909,9 +4924,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F115" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F115" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G115" s="34" t="inlineStr">
+        <is>
+          <t>Itération 5 — moyen de paiement actif au checkout</t>
         </is>
       </c>
     </row>
@@ -4939,9 +4959,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F116" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F116" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G116" s="34" t="inlineStr">
+        <is>
+          <t>Itération 5 — création auto au premier accès</t>
         </is>
       </c>
     </row>
@@ -4969,9 +4994,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F117" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F117" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G117" s="34" t="inlineStr">
+        <is>
+          <t>Itération 5 — wallet commun au compte (multi-casquettes)</t>
         </is>
       </c>
     </row>
@@ -4999,9 +5029,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F118" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F118" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G118" s="34" t="inlineStr">
+        <is>
+          <t>Itération 5</t>
         </is>
       </c>
     </row>
@@ -5029,9 +5064,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F119" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F119" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G119" s="34" t="inlineStr">
+        <is>
+          <t>Itération 5 — grand livre complet</t>
         </is>
       </c>
     </row>
@@ -5059,9 +5099,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F120" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F120" s="35" t="inlineStr">
+        <is>
+          <t>🟡 Partiel</t>
+        </is>
+      </c>
+      <c r="G120" s="34" t="inlineStr">
+        <is>
+          <t>Simulée en local ; agrégateur réel à brancher</t>
         </is>
       </c>
     </row>
@@ -5089,9 +5134,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F121" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F121" s="35" t="inlineStr">
+        <is>
+          <t>🟡 Partiel</t>
+        </is>
+      </c>
+      <c r="G121" s="34" t="inlineStr">
+        <is>
+          <t>Simulé en local ; agrégateur réel à brancher</t>
         </is>
       </c>
     </row>
@@ -5119,9 +5169,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F122" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F122" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G122" s="34" t="inlineStr">
+        <is>
+          <t>Itération 5 — commission 5 % au versement vendeur</t>
         </is>
       </c>
     </row>
@@ -5149,9 +5204,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F123" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F123" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G123" s="34" t="inlineStr">
+        <is>
+          <t>Itération 5</t>
         </is>
       </c>
     </row>
@@ -5179,9 +5239,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F124" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F124" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G124" s="34" t="inlineStr">
+        <is>
+          <t>Itération 5 — rien n'est versé avant confirmation</t>
         </is>
       </c>
     </row>
@@ -5209,9 +5274,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F125" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F125" s="35" t="inlineStr">
+        <is>
+          <t>🟡 Partiel</t>
+        </is>
+      </c>
+      <c r="G125" s="34" t="inlineStr">
+        <is>
+          <t>Visible dans l'espace vendeur ; notification au module Communication</t>
         </is>
       </c>
     </row>
@@ -5239,9 +5309,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F126" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F126" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G126" s="34" t="inlineStr">
+        <is>
+          <t>Itération 5 — à la confirmation de réception</t>
         </is>
       </c>
     </row>
@@ -5329,9 +5404,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F129" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F129" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G129" s="34" t="inlineStr">
+        <is>
+          <t>Itération 5 — net de commission</t>
         </is>
       </c>
     </row>
@@ -5479,9 +5559,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F134" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F134" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G134" s="34" t="inlineStr">
+        <is>
+          <t>Itération 5 — annulation avant expédition : remboursement + re-stock</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Suivi : iteration 6 marquee dans l explosion du projet
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Explosion du projet - MAJ.xlsx
+++ b/docs/Explosion du projet - MAJ.xlsx
@@ -5696,9 +5696,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F139" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F139" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G139" s="34" t="inlineStr">
+        <is>
+          <t>Itérations 4-5</t>
         </is>
       </c>
     </row>
@@ -5726,9 +5731,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F140" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F140" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G140" s="34" t="inlineStr">
+        <is>
+          <t>Itération 5</t>
         </is>
       </c>
     </row>
@@ -5786,9 +5796,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F142" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F142" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G142" s="34" t="inlineStr">
+        <is>
+          <t>Itération 5</t>
         </is>
       </c>
     </row>
@@ -5846,9 +5861,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F144" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F144" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G144" s="34" t="inlineStr">
+        <is>
+          <t>Itérations 5-6 — automatique à la récupération du colis</t>
         </is>
       </c>
     </row>
@@ -5906,9 +5926,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F146" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F146" s="35" t="inlineStr">
+        <is>
+          <t>🟡 Partiel</t>
+        </is>
+      </c>
+      <c r="G146" s="34" t="inlineStr">
+        <is>
+          <t>Itération 6 — suivi via la course (récupéré/remis) ; le statut commande reste « Expédiée »</t>
         </is>
       </c>
     </row>
@@ -5936,9 +5961,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F147" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F147" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G147" s="34" t="inlineStr">
+        <is>
+          <t>Itération 5</t>
         </is>
       </c>
     </row>
@@ -5966,9 +5996,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F148" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F148" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G148" s="34" t="inlineStr">
+        <is>
+          <t>Itération 5 — fonds versés à la confirmation de réception</t>
         </is>
       </c>
     </row>
@@ -5996,9 +6031,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F149" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F149" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G149" s="34" t="inlineStr">
+        <is>
+          <t>Itération 5</t>
         </is>
       </c>
     </row>
@@ -6026,9 +6066,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F150" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F150" s="35" t="inlineStr">
+        <is>
+          <t>🟡 Partiel</t>
+        </is>
+      </c>
+      <c r="G150" s="34" t="inlineStr">
+        <is>
+          <t>Remboursement wallet effectué ; le statut affiché reste « Annulée »</t>
         </is>
       </c>
     </row>
@@ -6176,9 +6221,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F155" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F155" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G155" s="34" t="inlineStr">
+        <is>
+          <t>Itération 5</t>
         </is>
       </c>
     </row>
@@ -6356,9 +6406,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F161" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F161" s="35" t="inlineStr">
+        <is>
+          <t>🟡 Partiel</t>
+        </is>
+      </c>
+      <c r="G161" s="34" t="inlineStr">
+        <is>
+          <t>Itération 6 — suivi sur le détail commande, pas de temps réel</t>
         </is>
       </c>
     </row>
@@ -6476,9 +6531,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F165" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F165" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G165" s="34" t="inlineStr">
+        <is>
+          <t>Itération 5</t>
         </is>
       </c>
     </row>
@@ -6566,9 +6626,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F168" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F168" s="35" t="inlineStr">
+        <is>
+          <t>🟡 Partiel</t>
+        </is>
+      </c>
+      <c r="G168" s="34" t="inlineStr">
+        <is>
+          <t>Itération 6 — timeline de la course ; timeline complète des statuts à venir</t>
         </is>
       </c>
     </row>
@@ -6686,9 +6751,14 @@
           <t>Moyenne</t>
         </is>
       </c>
-      <c r="F172" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F172" s="35" t="inlineStr">
+        <is>
+          <t>🟡 Partiel</t>
+        </is>
+      </c>
+      <c r="G172" s="34" t="inlineStr">
+        <is>
+          <t>Itération 6 — dates clés de la course</t>
         </is>
       </c>
     </row>
@@ -6716,9 +6786,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F173" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F173" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G173" s="34" t="inlineStr">
+        <is>
+          <t>Itération 6 — photo de preuve de remise</t>
         </is>
       </c>
     </row>
@@ -6758,9 +6833,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F175" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F175" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G175" s="34" t="inlineStr">
+        <is>
+          <t>Itération 6 — livreurs locaux (modèle casquette livreur)</t>
         </is>
       </c>
     </row>
@@ -6998,9 +7078,14 @@
           <t>Moyenne</t>
         </is>
       </c>
-      <c r="F183" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F183" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G183" s="34" t="inlineStr">
+        <is>
+          <t>Itération 4 — forfait provisoire 1 000 FCFA par vendeur</t>
         </is>
       </c>
     </row>
@@ -7028,9 +7113,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F184" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F184" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G184" s="34" t="inlineStr">
+        <is>
+          <t>Itération 4 — une commande et des frais par vendeur</t>
         </is>
       </c>
     </row>
@@ -7058,9 +7148,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F185" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F185" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G185" s="34" t="inlineStr">
+        <is>
+          <t>Itération 6</t>
         </is>
       </c>
     </row>
@@ -7118,9 +7213,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F187" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F187" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G187" s="34" t="inlineStr">
+        <is>
+          <t>Itération 6 — horodatage automatique</t>
         </is>
       </c>
     </row>
@@ -7148,9 +7248,14 @@
           <t>Moyenne</t>
         </is>
       </c>
-      <c r="F188" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F188" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G188" s="34" t="inlineStr">
+        <is>
+          <t>Itération 6</t>
         </is>
       </c>
     </row>
@@ -7178,9 +7283,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F189" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F189" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G189" s="34" t="inlineStr">
+        <is>
+          <t>Itération 6 — Storage privé + consultation à accès contrôlé</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Suivi : iteration 7 marquee dans l explosion du projet
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Explosion du projet - MAJ.xlsx
+++ b/docs/Explosion du projet - MAJ.xlsx
@@ -6066,14 +6066,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F150" s="35" t="inlineStr">
-        <is>
-          <t>🟡 Partiel</t>
+      <c r="F150" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
         </is>
       </c>
       <c r="G150" s="34" t="inlineStr">
         <is>
-          <t>Remboursement wallet effectué ; le statut affiché reste « Annulée »</t>
+          <t>Itérations 5-7 — statut « Remboursée » après litige ; remboursement aussi à l'annulation</t>
         </is>
       </c>
     </row>
@@ -6101,9 +6101,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F151" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F151" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G151" s="34" t="inlineStr">
+        <is>
+          <t>Itération 7 — blocage Escrow automatique</t>
         </is>
       </c>
     </row>
@@ -6566,9 +6571,14 @@
           <t>Moyenne</t>
         </is>
       </c>
-      <c r="F166" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F166" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G166" s="34" t="inlineStr">
+        <is>
+          <t>Itération 5 — annulation directe avant expédition</t>
         </is>
       </c>
     </row>
@@ -6596,9 +6606,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F167" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F167" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G167" s="34" t="inlineStr">
+        <is>
+          <t>Itération 7</t>
         </is>
       </c>
     </row>
@@ -7318,9 +7333,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F190" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F190" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G190" s="34" t="inlineStr">
+        <is>
+          <t>Itération 7 — motif de litige</t>
         </is>
       </c>
     </row>
@@ -7348,9 +7368,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F191" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F191" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G191" s="34" t="inlineStr">
+        <is>
+          <t>Itération 7 — motif de litige</t>
         </is>
       </c>
     </row>
@@ -7378,9 +7403,14 @@
           <t>Moyenne</t>
         </is>
       </c>
-      <c r="F192" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F192" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G192" s="34" t="inlineStr">
+        <is>
+          <t>Itération 7 — motif de litige</t>
         </is>
       </c>
     </row>
@@ -7408,9 +7438,14 @@
           <t>Moyenne</t>
         </is>
       </c>
-      <c r="F193" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F193" s="35" t="inlineStr">
+        <is>
+          <t>🟡 Partiel</t>
+        </is>
+      </c>
+      <c r="G193" s="34" t="inlineStr">
+        <is>
+          <t>Couvert par le motif « Autre problème »</t>
         </is>
       </c>
     </row>
@@ -7438,9 +7473,14 @@
           <t>Moyenne</t>
         </is>
       </c>
-      <c r="F194" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F194" s="35" t="inlineStr">
+        <is>
+          <t>🟡 Partiel</t>
+        </is>
+      </c>
+      <c r="G194" s="34" t="inlineStr">
+        <is>
+          <t>Couvert par le motif « Autre problème »</t>
         </is>
       </c>
     </row>
@@ -7510,9 +7550,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F197" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F197" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G197" s="34" t="inlineStr">
+        <is>
+          <t>Itération 7 — /compte/commandes/[id]/litige</t>
         </is>
       </c>
     </row>
@@ -7540,9 +7585,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F198" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F198" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G198" s="34" t="inlineStr">
+        <is>
+          <t>Itération 7 — 6 motifs</t>
         </is>
       </c>
     </row>
@@ -7570,9 +7620,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F199" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F199" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G199" s="34" t="inlineStr">
+        <is>
+          <t>Itération 7 — description obligatoire (20 caractères min)</t>
         </is>
       </c>
     </row>
@@ -7600,9 +7655,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F200" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F200" s="35" t="inlineStr">
+        <is>
+          <t>🟡 Partiel</t>
+        </is>
+      </c>
+      <c r="G200" s="34" t="inlineStr">
+        <is>
+          <t>Itération 7 — photos (4 max) ; vidéos à venir</t>
         </is>
       </c>
     </row>
@@ -7630,9 +7690,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F201" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F201" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G201" s="34" t="inlineStr">
+        <is>
+          <t>Itération 7 — commande « disputed », fonds gelés jusqu'à l'arbitrage</t>
         </is>
       </c>
     </row>
@@ -7660,9 +7725,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F202" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F202" s="35" t="inlineStr">
+        <is>
+          <t>🟡 Partiel</t>
+        </is>
+      </c>
+      <c r="G202" s="34" t="inlineStr">
+        <is>
+          <t>Litige visible sur les commandes vendeur ; notification au module Communication</t>
         </is>
       </c>
     </row>
@@ -7690,9 +7760,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F203" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F203" s="35" t="inlineStr">
+        <is>
+          <t>🟡 Partiel</t>
+        </is>
+      </c>
+      <c r="G203" s="34" t="inlineStr">
+        <is>
+          <t>Dashboard /admin/litiges ; notification au module Communication</t>
         </is>
       </c>
     </row>
@@ -7750,9 +7825,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F205" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F205" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G205" s="34" t="inlineStr">
+        <is>
+          <t>Itération 7 — litiges ouverts d'abord, total Escrow bloqué</t>
         </is>
       </c>
     </row>
@@ -7780,9 +7860,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F206" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F206" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G206" s="34" t="inlineStr">
+        <is>
+          <t>Itération 7 — page /litiges/[id]</t>
         </is>
       </c>
     </row>
@@ -7810,9 +7895,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F207" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F207" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G207" s="34" t="inlineStr">
+        <is>
+          <t>Itération 7 — fil d'échanges sur le litige</t>
         </is>
       </c>
     </row>
@@ -7840,9 +7930,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F208" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F208" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G208" s="34" t="inlineStr">
+        <is>
+          <t>Itération 7 — preuves consultables (accès contrôlé)</t>
         </is>
       </c>
     </row>
@@ -7870,9 +7965,14 @@
           <t>Moyenne</t>
         </is>
       </c>
-      <c r="F209" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F209" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G209" s="34" t="inlineStr">
+        <is>
+          <t>Itération 7 — via le fil d'échanges</t>
         </is>
       </c>
     </row>
@@ -7900,9 +8000,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F210" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F210" s="35" t="inlineStr">
+        <is>
+          <t>🟡 Partiel</t>
+        </is>
+      </c>
+      <c r="G210" s="34" t="inlineStr">
+        <is>
+          <t>Via le fil d'échanges ; proposition formalisée à venir</t>
         </is>
       </c>
     </row>
@@ -7930,9 +8035,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F211" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F211" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G211" s="34" t="inlineStr">
+        <is>
+          <t>Itération 7 — décision motivée (note visible par les parties)</t>
         </is>
       </c>
     </row>
@@ -7960,9 +8070,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F212" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F212" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G212" s="34" t="inlineStr">
+        <is>
+          <t>Itération 7 — total, partiel (solde au vendeur) ou rejet</t>
         </is>
       </c>
     </row>
@@ -7990,9 +8105,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F213" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F213" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G213" s="34" t="inlineStr">
+        <is>
+          <t>Itération 7 — net de commission, livreur payé si course effectuée</t>
         </is>
       </c>
     </row>
@@ -8020,9 +8140,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F214" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F214" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G214" s="34" t="inlineStr">
+        <is>
+          <t>Itération 7 — clôture à la décision</t>
         </is>
       </c>
     </row>
@@ -8050,9 +8175,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F215" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F215" s="35" t="inlineStr">
+        <is>
+          <t>🟡 Partiel</t>
+        </is>
+      </c>
+      <c r="G215" s="34" t="inlineStr">
+        <is>
+          <t>Fil d'échanges ; délai 48 h non automatisé (module Communication)</t>
         </is>
       </c>
     </row>
@@ -8080,9 +8210,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F216" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F216" s="35" t="inlineStr">
+        <is>
+          <t>🟡 Partiel</t>
+        </is>
+      </c>
+      <c r="G216" s="34" t="inlineStr">
+        <is>
+          <t>Médiation via le fil ; délais non automatisés</t>
         </is>
       </c>
     </row>
@@ -8110,9 +8245,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F217" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F217" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G217" s="34" t="inlineStr">
+        <is>
+          <t>Itération 7</t>
         </is>
       </c>
     </row>
@@ -8140,9 +8280,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F218" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F218" s="35" t="inlineStr">
+        <is>
+          <t>🟡 Partiel</t>
+        </is>
+      </c>
+      <c r="G218" s="34" t="inlineStr">
+        <is>
+          <t>Décision et note visibles par les parties ; notification à venir</t>
         </is>
       </c>
     </row>
@@ -8170,9 +8315,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F219" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F219" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G219" s="34" t="inlineStr">
+        <is>
+          <t>Itération 7 — mouvements de fonds transactionnels</t>
         </is>
       </c>
     </row>
@@ -8332,9 +8482,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F225" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F225" s="35" t="inlineStr">
+        <is>
+          <t>🟡 Partiel</t>
+        </is>
+      </c>
+      <c r="G225" s="34" t="inlineStr">
+        <is>
+          <t>Via litige avant confirmation ; garantie post-livraison à définir</t>
         </is>
       </c>
     </row>
@@ -8362,9 +8517,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F226" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F226" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G226" s="34" t="inlineStr">
+        <is>
+          <t>Itérations 5-7 — fonds bloqués jusqu'à réception ou arbitrage</t>
         </is>
       </c>
     </row>
@@ -8434,9 +8594,14 @@
           <t>Moyenne</t>
         </is>
       </c>
-      <c r="F229" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F229" s="35" t="inlineStr">
+        <is>
+          <t>🟡 Partiel</t>
+        </is>
+      </c>
+      <c r="G229" s="34" t="inlineStr">
+        <is>
+          <t>Itération 7 — limité au cadre du litige</t>
         </is>
       </c>
     </row>
@@ -8464,9 +8629,14 @@
           <t>Moyenne</t>
         </is>
       </c>
-      <c r="F230" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F230" s="35" t="inlineStr">
+        <is>
+          <t>🟡 Partiel</t>
+        </is>
+      </c>
+      <c r="G230" s="34" t="inlineStr">
+        <is>
+          <t>Itération 7 — limité au cadre du litige</t>
         </is>
       </c>
     </row>
@@ -8494,9 +8664,14 @@
           <t>Moyenne</t>
         </is>
       </c>
-      <c r="F231" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F231" s="35" t="inlineStr">
+        <is>
+          <t>🟡 Partiel</t>
+        </is>
+      </c>
+      <c r="G231" s="34" t="inlineStr">
+        <is>
+          <t>Itération 7 — limité au cadre du litige</t>
         </is>
       </c>
     </row>
@@ -8524,9 +8699,14 @@
           <t>Moyenne</t>
         </is>
       </c>
-      <c r="F232" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F232" s="35" t="inlineStr">
+        <is>
+          <t>🟡 Partiel</t>
+        </is>
+      </c>
+      <c r="G232" s="34" t="inlineStr">
+        <is>
+          <t>Itération 7 — fil de litige conservé</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Suivi : iteration 9 marquee dans l explosion du projet
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Explosion du projet - MAJ.xlsx
+++ b/docs/Explosion du projet - MAJ.xlsx
@@ -1444,9 +1444,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F9" s="35" t="inlineStr">
+        <is>
+          <t>🟡 Partiel</t>
+        </is>
+      </c>
+      <c r="G9" s="34" t="inlineStr">
+        <is>
+          <t>Itération 9 — lien envoyé + rappel/renvoi ; sans blocage fonctionnel</t>
         </is>
       </c>
     </row>
@@ -1849,9 +1854,14 @@
           <t>Moyenne</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F21" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G21" s="34" t="inlineStr">
+        <is>
+          <t>Itération 9 — cloche avec compteur + page notifications</t>
         </is>
       </c>
     </row>
@@ -2104,9 +2114,14 @@
           <t>Moyenne</t>
         </is>
       </c>
-      <c r="F29" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F29" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G29" s="34" t="inlineStr">
+        <is>
+          <t>Itération 9 — notifications vendeur (commandes, courses, litiges)</t>
         </is>
       </c>
     </row>
@@ -6141,9 +6156,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F152" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F152" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G152" s="34" t="inlineStr">
+        <is>
+          <t>Itération 9 — in-app + email</t>
         </is>
       </c>
     </row>
@@ -6171,9 +6191,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F153" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F153" s="35" t="inlineStr">
+        <is>
+          <t>🟡 Partiel</t>
+        </is>
+      </c>
+      <c r="G153" s="34" t="inlineStr">
+        <is>
+          <t>La préparation vaut acceptation ; refus avec motif à venir</t>
         </is>
       </c>
     </row>
@@ -6386,9 +6411,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F160" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F160" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G160" s="34" t="inlineStr">
+        <is>
+          <t>Itération 9</t>
         </is>
       </c>
     </row>
@@ -6681,9 +6711,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F169" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F169" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G169" s="34" t="inlineStr">
+        <is>
+          <t>Itération 9 — Brevo en prod, simulé en local (email_outbox)</t>
         </is>
       </c>
     </row>
@@ -7513,9 +7548,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F195" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F195" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G195" s="34" t="inlineStr">
+        <is>
+          <t>Itération 9 — refus de course, litiges, annulations notifiés</t>
         </is>
       </c>
     </row>
@@ -7730,14 +7770,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F202" s="35" t="inlineStr">
-        <is>
-          <t>🟡 Partiel</t>
+      <c r="F202" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
         </is>
       </c>
       <c r="G202" s="34" t="inlineStr">
         <is>
-          <t>Litige visible sur les commandes vendeur ; notification au module Communication</t>
+          <t>Itération 9 — in-app + email à l'ouverture</t>
         </is>
       </c>
     </row>
@@ -7765,14 +7805,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F203" s="35" t="inlineStr">
-        <is>
-          <t>🟡 Partiel</t>
+      <c r="F203" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
         </is>
       </c>
       <c r="G203" s="34" t="inlineStr">
         <is>
-          <t>Dashboard /admin/litiges ; notification au module Communication</t>
+          <t>Itération 9 — tous les admins notifiés</t>
         </is>
       </c>
     </row>
@@ -8285,14 +8325,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F218" s="35" t="inlineStr">
-        <is>
-          <t>🟡 Partiel</t>
+      <c r="F218" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
         </is>
       </c>
       <c r="G218" s="34" t="inlineStr">
         <is>
-          <t>Décision et note visibles par les parties ; notification à venir</t>
+          <t>Itération 9 — décision notifiée aux deux parties (in-app + email)</t>
         </is>
       </c>
     </row>
@@ -8754,9 +8794,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F233" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F233" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G233" s="34" t="inlineStr">
+        <is>
+          <t>Itération 9 — messages de litige notifiés aux autres parties</t>
         </is>
       </c>
     </row>
@@ -8784,9 +8829,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F234" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F234" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G234" s="34" t="inlineStr">
+        <is>
+          <t>Itération 9 — Brevo (simulé en local), journal email_outbox</t>
         </is>
       </c>
     </row>
@@ -11504,9 +11554,14 @@
           <t>Moyenne</t>
         </is>
       </c>
-      <c r="F320" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F320" s="35" t="inlineStr">
+        <is>
+          <t>🟡 Partiel</t>
+        </is>
+      </c>
+      <c r="G320" s="34" t="inlineStr">
+        <is>
+          <t>Demandes vendeur dans les tâches en attente admin ; notification à l'inscription à venir</t>
         </is>
       </c>
     </row>
@@ -11534,9 +11589,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F321" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F321" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G321" s="34" t="inlineStr">
+        <is>
+          <t>Itération 9 — in-app + email</t>
         </is>
       </c>
     </row>
@@ -11564,9 +11624,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F322" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F322" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G322" s="34" t="inlineStr">
+        <is>
+          <t>Itération 9 — in-app + email</t>
         </is>
       </c>
     </row>
@@ -11594,9 +11659,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F323" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F323" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G323" s="34" t="inlineStr">
+        <is>
+          <t>Itération 9 — expédition vendeur et récupération livreur</t>
         </is>
       </c>
     </row>
@@ -11624,9 +11694,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F324" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F324" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G324" s="34" t="inlineStr">
+        <is>
+          <t>Itération 9 — versements vendeur et livreur notifiés</t>
         </is>
       </c>
     </row>
@@ -11654,9 +11729,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F325" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F325" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G325" s="34" t="inlineStr">
+        <is>
+          <t>Itération 9 — fil de litige</t>
         </is>
       </c>
     </row>
@@ -11684,9 +11764,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F326" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F326" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G326" s="34" t="inlineStr">
+        <is>
+          <t>Itération 9 — vendeur + admins</t>
         </is>
       </c>
     </row>
@@ -11714,9 +11799,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F327" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F327" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G327" s="34" t="inlineStr">
+        <is>
+          <t>Itération 9 — les deux parties + livreur le cas échéant</t>
         </is>
       </c>
     </row>
@@ -11744,9 +11834,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F328" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F328" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G328" s="34" t="inlineStr">
+        <is>
+          <t>Itération 9 — approbation et refus, vendeur et livreur</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Suivi : iteration 10 marquee dans l explosion du projet
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Explosion du projet - MAJ.xlsx
+++ b/docs/Explosion du projet - MAJ.xlsx
@@ -5364,9 +5364,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F127" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F127" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G127" s="34" t="inlineStr">
+        <is>
+          <t>Itération 10 — 7 jours après expédition ; cron quotidien (Vercel Cron) + filet admin</t>
         </is>
       </c>
     </row>
@@ -5394,9 +5399,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F128" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F128" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G128" s="34" t="inlineStr">
+        <is>
+          <t>Itération 7 — remboursement total ou partiel sur arbitrage</t>
         </is>
       </c>
     </row>
@@ -5459,9 +5469,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F130" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F130" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G130" s="34" t="inlineStr">
+        <is>
+          <t>Itération 10 — PDF généré à la volée (pdf-lib)</t>
         </is>
       </c>
     </row>
@@ -5489,9 +5504,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F131" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F131" s="35" t="inlineStr">
+        <is>
+          <t>🟡 Partiel</t>
+        </is>
+      </c>
+      <c r="G131" s="34" t="inlineStr">
+        <is>
+          <t>Itération 10 — reçu email avec lien facture ; PDF joint à venir</t>
         </is>
       </c>
     </row>
@@ -5519,9 +5539,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F132" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F132" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G132" s="34" t="inlineStr">
+        <is>
+          <t>Itération 10 — /api/factures/[orderId], accès acheteur/vendeur/admin</t>
         </is>
       </c>
     </row>
@@ -5549,9 +5574,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F133" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F133" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G133" s="34" t="inlineStr">
+        <is>
+          <t>Itérations 5-8 — annulation, litige et intervention admin</t>
         </is>
       </c>
     </row>
@@ -6511,9 +6541,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F163" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F163" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G163" s="34" t="inlineStr">
+        <is>
+          <t>Itération 10 — bouton sur le détail de commande</t>
         </is>
       </c>
     </row>
@@ -10556,9 +10591,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F286" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F286" s="35" t="inlineStr">
+        <is>
+          <t>🟡 Partiel</t>
+        </is>
+      </c>
+      <c r="G286" s="34" t="inlineStr">
+        <is>
+          <t>Constante ESCROW_AUTO_RELEASE_DAYS (7 j) ; paramétrage en BDD à venir</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: suivi projet — promos/bannières/similaires marqués, feuille Suivi technique
8 statuts mis à jour (4 Réalisé, 3 Partiel honnêtes, SSL/TLS réalisé) et
nouvelle feuille « Suivi technique » : 10 travaux hors cahier livrés
(VPS, SMS, vitrine…) + 10 à faire (SSH, FedaPay, Brevo, backups…).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Explosion du projet - MAJ.xlsx
+++ b/docs/Explosion du projet - MAJ.xlsx
@@ -11,6 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 3" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fonctionnalités Marketplace" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suivi technique" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -212,7 +213,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -306,6 +307,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5646,7 +5648,12 @@
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>HTTPS Let's Encrypt automatique (Caddy) sur deallome.com — 2026-07-06</t>
         </is>
       </c>
     </row>
@@ -11885,8 +11892,6 @@
         </is>
       </c>
     </row>
-    <row r="329"/>
-    <row r="330"/>
     <row r="331" ht="16.3" customHeight="1" s="18">
       <c r="A331" s="24" t="inlineStr">
         <is>
@@ -12811,7 +12816,12 @@
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Prix barré + badge −% sur cartes et fiche — 2026-07-07</t>
         </is>
       </c>
     </row>
@@ -12871,7 +12881,12 @@
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>🟡 Partiel</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Échéance avec compte à rebours ; pas de date de début programmable</t>
         </is>
       </c>
     </row>
@@ -13903,7 +13918,12 @@
       </c>
       <c r="F67" s="4" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Fiche produit : « Produits similaires » (même rayon) — 2026-07-07</t>
         </is>
       </c>
     </row>
@@ -13933,7 +13953,12 @@
       </c>
       <c r="F68" s="4" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>🟡 Partiel</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>« Du même vendeur » sur la fiche ; pas d'algorithme personnalisé</t>
         </is>
       </c>
     </row>
@@ -17641,7 +17666,12 @@
       </c>
       <c r="F197" s="4" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G197" t="inlineStr">
+        <is>
+          <t>Carrousel de bannières produits sur l'accueil — 2026-07-07</t>
         </is>
       </c>
     </row>
@@ -17671,7 +17701,12 @@
       </c>
       <c r="F198" s="4" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G198" t="inlineStr">
+        <is>
+          <t>Section « Offres &amp; promos » avec compte à rebours — 2026-07-07</t>
         </is>
       </c>
     </row>
@@ -19105,7 +19140,12 @@
       </c>
       <c r="F247" s="4" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>🟡 Partiel</t>
+        </is>
+      </c>
+      <c r="G247" t="inlineStr">
+        <is>
+          <t>Promos à échéance + countdown ; pas de mécanique flash dédiée</t>
         </is>
       </c>
     </row>
@@ -41960,4 +42000,530 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" style="18" min="1" max="1"/>
+    <col width="16" customWidth="1" style="18" min="2" max="2"/>
+    <col width="72" customWidth="1" style="18" min="3" max="3"/>
+    <col width="12" customWidth="1" style="18" min="4" max="4"/>
+    <col width="62" customWidth="1" style="18" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="37" t="inlineStr">
+        <is>
+          <t>SUIVI TECHNIQUE — TRAVAUX HORS CAHIER DES CHARGES (MAJ 2026-07-07)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="36" t="inlineStr">
+        <is>
+          <t>N°</t>
+        </is>
+      </c>
+      <c r="B2" s="36" t="inlineStr">
+        <is>
+          <t>Domaine</t>
+        </is>
+      </c>
+      <c r="C2" s="36" t="inlineStr">
+        <is>
+          <t>Sujet</t>
+        </is>
+      </c>
+      <c r="D2" s="36" t="inlineStr">
+        <is>
+          <t>Statut</t>
+        </is>
+      </c>
+      <c r="E2" s="36" t="inlineStr">
+        <is>
+          <t>Commentaire</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Déploiement production VPS (Docker : PostgreSQL + app + Caddy)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>deallome.com en ligne (HTTPS) — 2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>DNS deallome.com + www → VPS, certificat TLS automatique</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Crons prod : déblocage Escrow (6h) + sauvegarde pg_dump (3h, rotation 7 j)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Runbook de déploiement (docs/DEPLOIEMENT.md)</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Routine + migrations + rollback + diagnostic</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Authentification</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Firebase Auth prod : email + téléphone, SMS réels vers le Togo</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Blocage anti-fraude Google levé via défense SMS reCAPTCHA (mode AUDIT)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Authentification</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Renvoi de code OTP avec cooldown + expiration affichée</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>UI/UX</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Vitrine marketplace (rampe catégories, rayons, carrousel héro)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Refonte orientée consommateur</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>UI/UX</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Écrans d'authentification en split + espace compte avec sidebar</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>UI/UX</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Header en icônes (Heroicons), footer global, police Bricolage Grotesque</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Données</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Catalogue de démonstration : 5 boutiques, 35 produits, 67 images, 7 promos</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Retirer au lancement : DELETE FROM users WHERE firebase_uid LIKE 'demo-seller-%'</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>11</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Sécurité</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Durcissement SSH du VPS (désactiver root + mot de passe)</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>À faire</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Accès par clé déjà en place</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>12</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Sécurité</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Rotation du mot de passe root du VPS</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>À faire</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Sécurité</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Sauvegardes externalisées chiffrées (Backblaze B2 / Object Storage)</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>À faire</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Obligatoire avant argent réel (cf. STACK.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>14</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Paiements</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Intégration agrégateur réel (FedaPay/CinetPay) et retrait de DEMO_MODE</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>À faire</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Recharges/retraits wallet actuellement simulés</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>15</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Emails</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Clé BREVO_API_KEY en prod (emails réels, domaine à authentifier SPF/DKIM)</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>À faire</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Emails journalisés « simulated » en attendant</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>16</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Vendeur</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Champs promo (prix promo + échéance) dans le formulaire produit vendeur</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>À faire</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Promos actuellement posées en base uniquement</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>UI/UX</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Migrer les icônes maison restantes (espace compte, auth) vers Heroicons</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>À faire</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>18</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Technique</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Self-host des polices (retour à next/font) quand le réseau build est stable</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>À faire</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>19</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Finances</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Alerte de budget GCP (coût des SMS)</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>À faire</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>~0,05 $/SMS au-delà de 10/jour</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>20</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Données</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Retrait du catalogue de démonstration au lancement commercial</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>À faire</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs(suivi): MAJ Excel - profil, boutique/logo, emails Brevo, panier invité, suggestions, placements, loader/UX
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Explosion du projet - MAJ.xlsx
+++ b/docs/Explosion du projet - MAJ.xlsx
@@ -1623,7 +1623,12 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Édition du profil sur /compte/profil (nom, infos personnelles) - 2026-07-09</t>
         </is>
       </c>
     </row>
@@ -1718,12 +1723,12 @@
       </c>
       <c r="F17" s="35" t="inlineStr">
         <is>
-          <t>🟡 Partiel</t>
+          <t>✅ Réalisé</t>
         </is>
       </c>
       <c r="G17" s="34" t="inlineStr">
         <is>
-          <t>Page compte créée ; manque commandes/wallet</t>
+          <t>Aperçu compte : soldes, commandes, notifications, casquettes, accès profil</t>
         </is>
       </c>
     </row>
@@ -2600,12 +2605,12 @@
       </c>
       <c r="F44" s="35" t="inlineStr">
         <is>
-          <t>🟡 Partiel</t>
+          <t>✅ Réalisé</t>
         </is>
       </c>
       <c r="G44" s="34" t="inlineStr">
         <is>
-          <t>Statut + motif visibles dans l'espace vendeur ; email/SMS à venir</t>
+          <t>Email réel (Brevo) au vendeur à la validation/au rejet de la demande</t>
         </is>
       </c>
     </row>
@@ -2700,7 +2705,12 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Description boutique éditable depuis le profil vendeur</t>
         </is>
       </c>
     </row>
@@ -2760,7 +2770,12 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Coordonnées de contact de la boutique éditables (téléphone)</t>
         </is>
       </c>
     </row>
@@ -5298,12 +5313,12 @@
       </c>
       <c r="F125" s="35" t="inlineStr">
         <is>
-          <t>🟡 Partiel</t>
+          <t>✅ Réalisé</t>
         </is>
       </c>
       <c r="G125" s="34" t="inlineStr">
         <is>
-          <t>Visible dans l'espace vendeur ; notification au module Communication</t>
+          <t>Email (Brevo) au vendeur : paiement sécurisé reçu</t>
         </is>
       </c>
     </row>
@@ -5513,7 +5528,7 @@
       </c>
       <c r="G131" s="34" t="inlineStr">
         <is>
-          <t>Itération 10 — reçu email avec lien facture ; PDF joint à venir</t>
+          <t>Reçu de paiement envoyé par email (Brevo) ; PDF non encore attaché</t>
         </is>
       </c>
     </row>
@@ -5653,7 +5668,7 @@
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>HTTPS Let's Encrypt automatique (Caddy) sur deallome.com — 2026-07-06</t>
+          <t>HTTPS Let's Encrypt automatique (Caddy) sur deallome.com - 2026-07-06</t>
         </is>
       </c>
     </row>
@@ -8878,7 +8893,7 @@
       </c>
       <c r="G234" s="34" t="inlineStr">
         <is>
-          <t>Itération 9 — Brevo (simulé en local), journal email_outbox</t>
+          <t>Brevo en prod : emails HTML de marque sur TOUS les événements du cycle de vie</t>
         </is>
       </c>
     </row>
@@ -12102,7 +12117,7 @@
       </c>
       <c r="G5" s="34" t="inlineStr">
         <is>
-          <t>Google réalisé (itération 2 bis) ; Facebook à faire</t>
+          <t>Google : code + intégration déployés ; activer le fournisseur dans la console Firebase</t>
         </is>
       </c>
     </row>
@@ -12444,7 +12459,12 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Upload du logo de boutique dans /compte/profil (colonne logo_url) ; règles Storage à publier</t>
         </is>
       </c>
     </row>
@@ -12504,7 +12524,12 @@
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Section « À la une » + emplacements sponsorisés sur l'accueil</t>
         </is>
       </c>
     </row>
@@ -12821,7 +12846,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Prix barré + badge −% sur cartes et fiche — 2026-07-07</t>
+          <t>Prix barré + badge de remise sur cartes et fiche</t>
         </is>
       </c>
     </row>
@@ -13528,7 +13553,12 @@
       </c>
       <c r="F54" s="4" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Rayon de suggestions affiché sur une recherche sans résultat</t>
         </is>
       </c>
     </row>
@@ -13923,7 +13953,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Fiche produit : « Produits similaires » (même rayon) — 2026-07-07</t>
+          <t>Fiche produit : « Produits similaires » (même rayon)</t>
         </is>
       </c>
     </row>
@@ -14090,7 +14120,12 @@
       </c>
       <c r="F73" s="4" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>Panier en base (connecté) + panier invité en cookie, fusionné à la connexion</t>
         </is>
       </c>
     </row>
@@ -17671,7 +17706,7 @@
       </c>
       <c r="G197" t="inlineStr">
         <is>
-          <t>Carrousel de bannières produits sur l'accueil — 2026-07-07</t>
+          <t>Carrousel de bannières produits sur l'accueil</t>
         </is>
       </c>
     </row>
@@ -17706,7 +17741,7 @@
       </c>
       <c r="G198" t="inlineStr">
         <is>
-          <t>Section « Offres &amp; promos » avec compte à rebours — 2026-07-07</t>
+          <t>Section « Offres &amp; promos » (carrousel auto + compte à rebours)</t>
         </is>
       </c>
     </row>
@@ -19976,7 +20011,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F101"/>
+  <dimension ref="A1:G101"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.3"/>
   <cols>
     <col width="8" customWidth="1" style="18" min="1" max="1"/>
@@ -20024,6 +20059,11 @@
           <t>Statut</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Commentaire</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="16.3" customHeight="1" s="18">
       <c r="A3" s="23" t="inlineStr">
@@ -20861,7 +20901,12 @@
       </c>
       <c r="F33" s="6" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Rayon « Continuez vos achats » sous le panier rempli (hors articles déjà au panier)</t>
         </is>
       </c>
     </row>
@@ -42008,20 +42053,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" style="18" min="1" max="1"/>
     <col width="16" customWidth="1" style="18" min="2" max="2"/>
-    <col width="72" customWidth="1" style="18" min="3" max="3"/>
+    <col width="78" customWidth="1" style="18" min="3" max="3"/>
     <col width="12" customWidth="1" style="18" min="4" max="4"/>
-    <col width="62" customWidth="1" style="18" min="5" max="5"/>
+    <col width="66" customWidth="1" style="18" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="37" t="inlineStr">
         <is>
-          <t>SUIVI TECHNIQUE — TRAVAUX HORS CAHIER DES CHARGES (MAJ 2026-07-07)</t>
+          <t>SUIVI TECHNIQUE - TRAVAUX HORS CAHIER DES CHARGES (MAJ 2026-07-10)</t>
         </is>
       </c>
     </row>
@@ -42073,7 +42118,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>deallome.com en ligne (HTTPS) — 2026-07-06</t>
+          <t>deallome.com en ligne (HTTPS) - 2026-07-06</t>
         </is>
       </c>
     </row>
@@ -42088,7 +42133,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>DNS deallome.com + www → VPS, certificat TLS automatique</t>
+          <t>DNS deallome.com + www vers le VPS, certificat TLS automatique</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -42165,7 +42210,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Blocage anti-fraude Google levé via défense SMS reCAPTCHA (mode AUDIT)</t>
+          <t>Blocage anti-fraude Google levé (défense SMS reCAPTCHA en mode AUDIT)</t>
         </is>
       </c>
     </row>
@@ -42188,11 +42233,7 @@
           <t>✅ Réalisé</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>2026-07-07</t>
-        </is>
-      </c>
+      <c r="E8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -42200,22 +42241,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>UI/UX</t>
+          <t>Authentification</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Vitrine marketplace (rampe catégories, rayons, carrousel héro)</t>
+          <t>Connexion / inscription Google (code + intégration déployés)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>✅ Réalisé</t>
+          <t>🟡 Partiel</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Refonte orientée consommateur</t>
+          <t>Activer le fournisseur Google dans la console Firebase pour l'utiliser</t>
         </is>
       </c>
     </row>
@@ -42225,12 +42266,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>UI/UX</t>
+          <t>Parcours d'achat</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Écrans d'authentification en split + espace compte avec sidebar</t>
+          <t>Achat invité : navigation et panier sans compte</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -42238,7 +42279,11 @@
           <t>✅ Réalisé</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Panier en cookie ; auth demandée uniquement au paiement</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -42246,12 +42291,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>UI/UX</t>
+          <t>Parcours d'achat</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Header en icônes (Heroicons), footer global, police Bricolage Grotesque</t>
+          <t>Fusion du panier invité dans le compte à la connexion</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -42259,7 +42304,11 @@
           <t>✅ Réalisé</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Plus de redirection brutale vers la connexion</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -42267,12 +42316,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Données</t>
+          <t>UI/UX</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Catalogue de démonstration : 5 boutiques, 35 produits, 67 images, 7 promos</t>
+          <t>Vitrine marketplace (rampe catégories, rayons, carrousel héro)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -42282,7 +42331,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Retirer au lancement : DELETE FROM users WHERE firebase_uid LIKE 'demo-seller-%'</t>
+          <t>Refonte orientée consommateur</t>
         </is>
       </c>
     </row>
@@ -42292,24 +42341,20 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Sécurité</t>
+          <t>UI/UX</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Durcissement SSH du VPS (désactiver root + mot de passe)</t>
+          <t>Écrans d'authentification en split + espace compte avec sidebar</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Accès par clé déjà en place</t>
-        </is>
-      </c>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -42317,20 +42362,24 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Sécurité</t>
+          <t>UI/UX</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Rotation du mot de passe root du VPS</t>
+          <t>Header en icônes (Heroicons) + menu déroulant « Mon espace »</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr"/>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Icône utilisateur, badges panier/notifications</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -42338,24 +42387,20 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Sécurité</t>
+          <t>UI/UX</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Sauvegardes externalisées chiffrées (Backblaze B2 / Object Storage)</t>
+          <t>Carrousel auto-défilant des « Offres &amp; promos »</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>Obligatoire avant argent réel (cf. STACK.md)</t>
-        </is>
-      </c>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -42363,22 +42408,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Paiements</t>
+          <t>UI/UX</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Intégration agrégateur réel (FedaPay/CinetPay) et retrait de DEMO_MODE</t>
+          <t>Suggestions produits (panier vide, panier rempli, recherche sans résultat)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Recharges/retraits wallet actuellement simulés</t>
+          <t>« inonder » l'utilisateur de produits</t>
         </is>
       </c>
     </row>
@@ -42388,22 +42433,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Emails</t>
+          <t>UI/UX</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Clé BREVO_API_KEY en prod (emails réels, domaine à authentifier SPF/DKIM)</t>
+          <t>Emplacements « À la une » + bandeaux promo maison in-feed</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Emails journalisés « simulated » en attendant</t>
+          <t>Placements natifs plutôt que pubs latérales ; badge « Sponsorisé » prêt</t>
         </is>
       </c>
     </row>
@@ -42413,22 +42458,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Vendeur</t>
+          <t>UI/UX</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Champs promo (prix promo + échéance) dans le formulaire produit vendeur</t>
+          <t>Loader : spinner boutons (soumissions/upload) + barre de progression de navigation (façon YouTube)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Promos actuellement posées en base uniquement</t>
+          <t>Barre confondue à la bordure du header</t>
         </is>
       </c>
     </row>
@@ -42443,12 +42488,12 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Migrer les icônes maison restantes (espace compte, auth) vers Heroicons</t>
+          <t>Bouton « retour en haut » + header masqué/révélé au scroll</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
         </is>
       </c>
       <c r="E19" t="inlineStr"/>
@@ -42459,20 +42504,24 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Technique</t>
+          <t>UI/UX</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Self-host des polices (retour à next/font) quand le réseau build est stable</t>
+          <t>Édition du profil : nom + boutique (nom, description, ville, quartier, tél, logo)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr"/>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Logo via Storage (règles à publier)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -42480,24 +42529,20 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Finances</t>
+          <t>UI/UX</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Alerte de budget GCP (coût des SMS)</t>
+          <t>Remplacement des flèches par des chevrons et des em-dashes par des tirets</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>~0,05 $/SMS au-delà de 10/jour</t>
-        </is>
-      </c>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -42505,20 +42550,312 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
+          <t>UI/UX</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Retrait du jargon « Escrow » au profit de « paiement sécurisé » (côté public)</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>21</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Emails</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Intégration Brevo en production</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Clé posée, domaine authentifié (DKIM/DMARC), IP autorisée, template HTML de marque</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>22</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Emails</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Emails transactionnels sur tous les événements du cycle de vie</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Commande, paiement, expédition, livraison, gains livreur, validations, litiges</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>23</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Emails</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Envoi de la facture PDF en pièce jointe</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>À faire</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Aujourd'hui : lien vers le détail de la commande</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>24</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Stockage</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Firebase Storage activé + CORS du bucket configuré</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Bucket deallome-staging.firebasestorage.app, origine deallome.com autorisée</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>25</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Stockage</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Règles de sécurité Storage (KYC privé, logos/produits publics)</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>À faire</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>À publier dans la console Firebase (fournies)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>26</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
           <t>Données</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Catalogue de démonstration : 5 boutiques, 63 produits, images</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Seed idempotent et non destructif ; retirer au lancement</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>27</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Sécurité</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Durcissement SSH du VPS (désactiver root + mot de passe)</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>À faire</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Accès par clé déjà en place</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>28</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Sécurité</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Rotation du mot de passe root du VPS</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>À faire</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>29</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Sécurité</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Sauvegardes externalisées chiffrées (Backblaze B2 / Object Storage)</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>À faire</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Obligatoire avant argent réel</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>30</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Paiements</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Intégration agrégateur réel (FedaPay/CinetPay) et retrait de DEMO_MODE</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>À faire</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Recharges/retraits wallet actuellement simulés</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>31</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Finances</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Alerte de budget GCP (coût des SMS)</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>À faire</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>~0,05 $/SMS au-delà de 10/jour</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>32</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Données</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
         <is>
           <t>Retrait du catalogue de démonstration au lancement commercial</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr"/>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>À faire</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
docs(suivi): MAJ Excel - cycle de commande vendeur (acceptation/refus, suivi, facture PDF)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Explosion du projet - MAJ.xlsx
+++ b/docs/Explosion du projet - MAJ.xlsx
@@ -5524,12 +5524,12 @@
       </c>
       <c r="F131" s="23" t="inlineStr">
         <is>
-          <t>🟡 Partiel</t>
+          <t>✅ Réalisé</t>
         </is>
       </c>
       <c r="G131" s="22" t="inlineStr">
         <is>
-          <t>Reçu de paiement envoyé par email (Brevo) ; PDF non encore attaché</t>
+          <t>Facture PDF jointe à l'email de confirmation de paiement (Brevo)</t>
         </is>
       </c>
     </row>
@@ -5841,7 +5841,12 @@
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>Acceptation vendeur (payée -&gt; en préparation) + notification acheteur</t>
         </is>
       </c>
     </row>
@@ -6246,12 +6251,12 @@
       </c>
       <c r="F153" s="23" t="inlineStr">
         <is>
-          <t>🟡 Partiel</t>
+          <t>✅ Réalisé</t>
         </is>
       </c>
       <c r="G153" s="22" t="inlineStr">
         <is>
-          <t>La préparation vaut acceptation ; refus avec motif à venir</t>
+          <t>Bouton « Accepter et préparer » ; l'acheteur est notifié de l'acceptation</t>
         </is>
       </c>
     </row>
@@ -6281,7 +6286,12 @@
       </c>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>Refus vendeur avec motif : remboursement + restitution du stock + notification</t>
         </is>
       </c>
     </row>
@@ -6376,7 +6386,12 @@
       </c>
       <c r="F157" s="2" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>Saisie n° de suivi + date estimée à l'expédition (auto-livraison)</t>
         </is>
       </c>
     </row>
@@ -6811,7 +6826,12 @@
       </c>
       <c r="F170" s="2" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>N° de suivi affiché sur le détail de commande de l'acheteur</t>
         </is>
       </c>
     </row>
@@ -6841,7 +6861,12 @@
       </c>
       <c r="F171" s="2" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>Date estimée de livraison affichée à l'acheteur</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(vendeur): onboarding & boutique - justificatif adresse, coordonnées de versement (Mobile Money/RIB), CGV vendeur, page boutique publique
- Candidature vendeur : upload justificatif d'adresse (optionnel) + acceptation obligatoire des conditions vendeur (page /cgv-vendeur)
- Profil vendeur : coordonnées de versement (Mobile Money Flooz/T-Money ou RIB/IBAN) + conditions de vente éditables
- Page boutique publique /boutique/[id] : logo, description, conditions de vente, catalogue ; liée depuis la fiche produit et l'espace vendeur
- Admin : justificatif d'adresse consultable + méthode de versement affichée
- Migration 0013 : colonnes seller_profiles (address_document_path, payout_*, bank_*, selling_conditions, terms_accepted_at)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Explosion du projet - MAJ.xlsx
+++ b/docs/Explosion du projet - MAJ.xlsx
@@ -2241,7 +2241,12 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Upload d'un justificatif d'adresse (optionnel) à la candidature vendeur ; consultable par l'admin</t>
         </is>
       </c>
     </row>
@@ -2341,7 +2346,12 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Coordonnées bancaires (banque, titulaire, RIB/IBAN) de versement dans le profil vendeur</t>
         </is>
       </c>
     </row>
@@ -2371,7 +2381,12 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Coordonnées Mobile Money (Flooz/T-Money) de versement dans le profil vendeur</t>
         </is>
       </c>
     </row>
@@ -2401,7 +2416,12 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Acceptation obligatoire des conditions vendeur (page /cgv-vendeur) à la candidature</t>
         </is>
       </c>
     </row>
@@ -2676,7 +2696,12 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Page boutique publique /boutique/[id] : logo, description, conditions de vente, catalogue</t>
         </is>
       </c>
     </row>
@@ -2741,7 +2766,12 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Conditions de vente de la boutique éditables (profil) et affichées sur la page publique</t>
         </is>
       </c>
     </row>
@@ -42697,12 +42727,12 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Aujourd'hui : lien vers le détail de la commande</t>
+          <t>Facture PDF attachée à l'email de confirmation de paiement (Brevo)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(suivi): MAJ Excel - promos vendeur (Phase 2 #25 réalisé, #26/#27 partiels) + navigation d'espaces et loader d'upload média (Suivi technique)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Explosion du projet - MAJ.xlsx
+++ b/docs/Explosion du projet - MAJ.xlsx
@@ -12942,7 +12942,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Prix barré + badge de remise sur cartes et fiche</t>
+          <t>Prix barré + badge de remise ; le vendeur définit le prix promo et l'échéance depuis la fiche produit</t>
         </is>
       </c>
     </row>
@@ -12972,7 +12972,12 @@
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>🟡 Partiel</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Badge -X% calculé et affiché ; le vendeur saisit un prix promo (montant), pas un pourcentage</t>
         </is>
       </c>
     </row>
@@ -13007,7 +13012,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Échéance avec compte à rebours ; pas de date de début programmable</t>
+          <t>Échéance de fin de promo éditable par le vendeur + compte à rebours ; pas de date de début programmable</t>
         </is>
       </c>
     </row>
@@ -42149,7 +42154,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" style="26" min="1" max="1"/>
@@ -42605,7 +42610,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Édition du profil : nom + boutique (nom, description, ville, quartier, tél, logo)</t>
+          <t>Navigation d'espace vendeur &amp; livreur (en-tête + onglets actifs) ; admin avec pastilles de tâches en attente</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -42615,7 +42620,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Logo via Storage (règles à publier)</t>
+          <t>Espaces vendeur/livreur jusque-là sans en-tête</t>
         </is>
       </c>
     </row>
@@ -42630,7 +42635,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Remplacement des flèches par des chevrons et des em-dashes par des tirets</t>
+          <t>Loader d'upload média avec progression réelle (% par photo + barre globale + spinner par vignette)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -42638,7 +42643,11 @@
           <t>✅ Réalisé</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Fin de l'écran figé au téléversement des photos produit</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -42651,7 +42660,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Retrait du jargon « Escrow » au profit de « paiement sécurisé » (côté public)</t>
+          <t>Édition du profil : nom + boutique (nom, description, ville, quartier, tél, logo)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -42659,7 +42668,11 @@
           <t>✅ Réalisé</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Logo via Storage (règles à publier)</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -42667,12 +42680,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Emails</t>
+          <t>UI/UX</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Intégration Brevo en production</t>
+          <t>Remplacement des flèches par des chevrons et des em-dashes par des tirets</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -42680,11 +42693,7 @@
           <t>✅ Réalisé</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>Clé posée, domaine authentifié (DKIM/DMARC), IP autorisée, template HTML de marque</t>
-        </is>
-      </c>
+      <c r="E23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -42692,12 +42701,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Emails</t>
+          <t>UI/UX</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Emails transactionnels sur tous les événements du cycle de vie</t>
+          <t>Retrait du jargon « Escrow » au profit de « paiement sécurisé » (côté public)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -42705,11 +42714,7 @@
           <t>✅ Réalisé</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>Commande, paiement, expédition, livraison, gains livreur, validations, litiges</t>
-        </is>
-      </c>
+      <c r="E24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -42722,7 +42727,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Envoi de la facture PDF en pièce jointe</t>
+          <t>Intégration Brevo en production</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -42732,7 +42737,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Facture PDF attachée à l'email de confirmation de paiement (Brevo)</t>
+          <t>Clé posée, domaine authentifié (DKIM/DMARC), IP autorisée, template HTML de marque</t>
         </is>
       </c>
     </row>
@@ -42742,12 +42747,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Stockage</t>
+          <t>Emails</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Firebase Storage activé + CORS du bucket configuré</t>
+          <t>Emails transactionnels sur tous les événements du cycle de vie</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -42757,7 +42762,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Bucket deallome-staging.firebasestorage.app, origine deallome.com autorisée</t>
+          <t>Commande, paiement, expédition, livraison, gains livreur, validations, litiges</t>
         </is>
       </c>
     </row>
@@ -42767,22 +42772,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Stockage</t>
+          <t>Emails</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Règles de sécurité Storage (KYC privé, logos/produits publics)</t>
+          <t>Envoi de la facture PDF en pièce jointe</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>À publier dans la console Firebase (fournies)</t>
+          <t>Facture PDF attachée à l'email de confirmation de paiement (Brevo)</t>
         </is>
       </c>
     </row>
@@ -42792,12 +42797,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Données</t>
+          <t>Stockage</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Catalogue de démonstration : 5 boutiques, 63 produits, images</t>
+          <t>Firebase Storage activé + CORS du bucket configuré</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -42807,7 +42812,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Seed idempotent et non destructif ; retirer au lancement</t>
+          <t>Bucket deallome-staging.firebasestorage.app, origine deallome.com autorisée</t>
         </is>
       </c>
     </row>
@@ -42817,12 +42822,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Sécurité</t>
+          <t>Stockage</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Durcissement SSH du VPS (désactiver root + mot de passe)</t>
+          <t>Règles de sécurité Storage (KYC privé, logos/produits publics)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -42832,7 +42837,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Accès par clé déjà en place</t>
+          <t>À publier dans la console Firebase (fournies)</t>
         </is>
       </c>
     </row>
@@ -42842,20 +42847,24 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Sécurité</t>
+          <t>Données</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Rotation du mot de passe root du VPS</t>
+          <t>Catalogue de démonstration : 5 boutiques, 63 produits, images</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr"/>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Seed idempotent et non destructif ; retirer au lancement</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -42868,7 +42877,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Sauvegardes externalisées chiffrées (Backblaze B2 / Object Storage)</t>
+          <t>Durcissement SSH du VPS (désactiver root + mot de passe)</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -42878,7 +42887,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Obligatoire avant argent réel</t>
+          <t>Accès par clé déjà en place</t>
         </is>
       </c>
     </row>
@@ -42888,12 +42897,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Paiements</t>
+          <t>Sécurité</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Intégration agrégateur réel (FedaPay/CinetPay) et retrait de DEMO_MODE</t>
+          <t>Rotation du mot de passe root du VPS</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -42901,11 +42910,7 @@
           <t>À faire</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>Recharges/retraits wallet actuellement simulés</t>
-        </is>
-      </c>
+      <c r="E32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -42913,12 +42918,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Finances</t>
+          <t>Sécurité</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Alerte de budget GCP (coût des SMS)</t>
+          <t>Sauvegardes externalisées chiffrées (Backblaze B2 / Object Storage)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -42928,7 +42933,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>~0,05 $/SMS au-delà de 10/jour</t>
+          <t>Obligatoire avant argent réel</t>
         </is>
       </c>
     </row>
@@ -42938,20 +42943,70 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
+          <t>Paiements</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Intégration agrégateur réel (FedaPay/CinetPay) et retrait de DEMO_MODE</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>À faire</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Recharges/retraits wallet actuellement simulés</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>33</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Finances</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Alerte de budget GCP (coût des SMS)</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>À faire</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>~0,05 $/SMS au-delà de 10/jour</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>34</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
           <t>Données</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>Retrait du catalogue de démonstration au lancement commercial</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr"/>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>À faire</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
docs(suivi): MAJ Excel - back-office admin (catégories #264-266, paramètres #267/270/271, journal #296, édition vendeur #241) + espaces unifiés
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Explosion du projet - MAJ.xlsx
+++ b/docs/Explosion du projet - MAJ.xlsx
@@ -9656,7 +9656,12 @@
       </c>
       <c r="F255" s="2" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G255" t="inlineStr">
+        <is>
+          <t>Modification des informations boutique par l'admin (journalisée)</t>
         </is>
       </c>
     </row>
@@ -10451,7 +10456,12 @@
       </c>
       <c r="F278" s="2" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G278" t="inlineStr">
+        <is>
+          <t>Création de catégories et sous-catégories dans /admin/categories (slug unique, 2 niveaux)</t>
         </is>
       </c>
     </row>
@@ -10481,7 +10491,12 @@
       </c>
       <c r="F279" s="2" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G279" t="inlineStr">
+        <is>
+          <t>Renommage des catégories (slug conservé, liens intacts)</t>
         </is>
       </c>
     </row>
@@ -10511,7 +10526,12 @@
       </c>
       <c r="F280" s="2" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G280" t="inlineStr">
+        <is>
+          <t>Suppression protégée : refusée si sous-catégories ou produits rattachés</t>
         </is>
       </c>
     </row>
@@ -10541,7 +10561,12 @@
       </c>
       <c r="F281" s="2" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G281" t="inlineStr">
+        <is>
+          <t>Page /admin/parametres : tarification éditable + configuration MVP affichée</t>
         </is>
       </c>
     </row>
@@ -10571,7 +10596,12 @@
       </c>
       <c r="F282" s="2" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>🟡 Partiel</t>
+        </is>
+      </c>
+      <c r="G282" t="inlineStr">
+        <is>
+          <t>Devise unique XOF (choix MVP), affichée dans les paramètres</t>
         </is>
       </c>
     </row>
@@ -10601,7 +10631,12 @@
       </c>
       <c r="F283" s="2" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>🟡 Partiel</t>
+        </is>
+      </c>
+      <c r="G283" t="inlineStr">
+        <is>
+          <t>Zone Lomé (MVP) affichée ; vraie gestion des zones au module livraison</t>
         </is>
       </c>
     </row>
@@ -10631,7 +10666,12 @@
       </c>
       <c r="F284" s="2" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G284" t="inlineStr">
+        <is>
+          <t>Taux de commission éditable, appliqué aux prochains versements vendeurs et arbitrages</t>
         </is>
       </c>
     </row>
@@ -10661,7 +10701,12 @@
       </c>
       <c r="F285" s="2" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t>Frais de livraison par vendeur éditables, appliqués au panier et au checkout</t>
         </is>
       </c>
     </row>
@@ -11485,7 +11530,12 @@
       </c>
       <c r="F312" s="2" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G312" t="inlineStr">
+        <is>
+          <t>Journal d'activité admin (/admin/journal) : validations, suspensions, arbitrages, catégories, paramètres</t>
         </is>
       </c>
     </row>
@@ -42610,7 +42660,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Navigation d'espace vendeur &amp; livreur (en-tête + onglets actifs) ; admin avec pastilles de tâches en attente</t>
+          <t>Espaces vendeur &amp; livreur unifiés dans la coquille compte (sidebar en groupes) ; admin avec en-tête dédié et pastilles de tâches</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -42620,7 +42670,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Espaces vendeur/livreur jusque-là sans en-tête</t>
+          <t>« Ma boutique » en nouvel onglet ; liens « devenir vendeur/livreur » discrets ; aperçu remodelé (chiffres clés + dernières commandes)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(suivi): MAJ Excel - dashboards & rapports (vendeur #20/21/24/25, analytics admin #278-283) + admin en sidebar
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Explosion du projet - MAJ.xlsx
+++ b/docs/Explosion du projet - MAJ.xlsx
@@ -1934,7 +1934,12 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Tableau de bord vendeur /vendeur : produits en ligne, commandes à accepter/en cours, CA net versé</t>
         </is>
       </c>
     </row>
@@ -1964,7 +1969,12 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Statistiques de ventes : commandes par statut + meilleures ventes (quantités et montants)</t>
         </is>
       </c>
     </row>
@@ -2064,7 +2074,12 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Gestion des produits /vendeur/produits : création, édition, publication, archivage, promo</t>
         </is>
       </c>
     </row>
@@ -2094,7 +2109,12 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Derniers versements sur le tableau de bord vendeur + historique complet dans le wallet</t>
         </is>
       </c>
     </row>
@@ -10936,7 +10956,12 @@
       </c>
       <c r="F292" s="2" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G292" t="inlineStr">
+        <is>
+          <t>Rapport ventes : commandes et volume d'affaires par mois (/admin/rapports)</t>
         </is>
       </c>
     </row>
@@ -10966,7 +10991,12 @@
       </c>
       <c r="F293" s="2" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G293" t="inlineStr">
+        <is>
+          <t>Rapport utilisateurs : inscriptions par mois</t>
         </is>
       </c>
     </row>
@@ -10996,7 +11026,12 @@
       </c>
       <c r="F294" s="2" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G294" t="inlineStr">
+        <is>
+          <t>Rapport vendeurs : boutiques les plus actives (commandes, volume)</t>
         </is>
       </c>
     </row>
@@ -11026,7 +11061,12 @@
       </c>
       <c r="F295" s="2" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G295" t="inlineStr">
+        <is>
+          <t>Rapport produits : meilleures ventes (quantités, montants)</t>
         </is>
       </c>
     </row>
@@ -11056,7 +11096,12 @@
       </c>
       <c r="F296" s="2" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G296" t="inlineStr">
+        <is>
+          <t>Rapport commissions : total perçu + détail par mois</t>
         </is>
       </c>
     </row>
@@ -11086,7 +11131,12 @@
       </c>
       <c r="F297" s="2" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G297" t="inlineStr">
+        <is>
+          <t>Rapport litiges : répartition par statut et motif, taux de litiges</t>
         </is>
       </c>
     </row>
@@ -42660,7 +42710,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Espaces vendeur &amp; livreur unifiés dans la coquille compte (sidebar en groupes) ; admin avec en-tête dédié et pastilles de tâches</t>
+          <t>Espaces vendeur &amp; livreur unifiés dans la coquille compte (sidebar en groupes) ; admin en sidebar dédiée (3 groupes) avec pastilles de tâches</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">

</xml_diff>

<commit_message>
docs(suivi): MAJ Excel - SEO (#289-291), signalements produits (#275), FAQ (#223)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Explosion du projet - MAJ.xlsx
+++ b/docs/Explosion du projet - MAJ.xlsx
@@ -9044,7 +9044,12 @@
       </c>
       <c r="F236" s="2" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G236" t="inlineStr">
+        <is>
+          <t>Page /faq en accordéons (commander, livraison, litiges, vendre, livrer, compte), reliée au footer</t>
         </is>
       </c>
     </row>
@@ -10856,7 +10861,12 @@
       </c>
       <c r="F289" s="2" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G289" t="inlineStr">
+        <is>
+          <t>Signalement produit sur la fiche (connecté) + examen admin : retrait du produit ou classement, journalisé</t>
         </is>
       </c>
     </row>
@@ -11355,7 +11365,12 @@
       </c>
       <c r="F305" s="2" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G305" t="inlineStr">
+        <is>
+          <t>URLs produit avec slug (/produits/slug-uuid), anciens liens redirigés en 308 vers l'URL canonique</t>
         </is>
       </c>
     </row>
@@ -11385,7 +11400,12 @@
       </c>
       <c r="F306" s="2" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G306" t="inlineStr">
+        <is>
+          <t>Méta-titres dynamiques : fiche produit (titre + prix), catalogue par rayon/recherche, boutique publique</t>
         </is>
       </c>
     </row>
@@ -11415,7 +11435,12 @@
       </c>
       <c r="F307" s="2" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G307" t="inlineStr">
+        <is>
+          <t>Méta-descriptions dynamiques (description produit tronquée ou repli boutique/plateforme)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(suivi): MAJ Excel - messagerie acheteur-vendeur (#150, #155)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Explosion du projet - MAJ.xlsx
+++ b/docs/Explosion du projet - MAJ.xlsx
@@ -6501,7 +6501,12 @@
       </c>
       <c r="F159" s="2" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>Vendeur : /vendeur/messages + « Contacter l'acheteur » depuis chaque commande, badges non-lus</t>
         </is>
       </c>
     </row>
@@ -6671,7 +6676,12 @@
       </c>
       <c r="F164" s="2" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>Acheteur : /compte/messages + « Contacter le vendeur » depuis la fiche produit et la commande, sujet prérempli</t>
         </is>
       </c>
     </row>

</xml_diff>